<commit_message>
Update example test file CFDataBarNegative
Update reference test file for example CFDataBarNegative. After style
infrastructure switch, the styles part is saved differently. No
semantic change to the styles part.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFDataBarNegative.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFDataBarNegative.xlsx
@@ -18,61 +18,52 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -408,7 +399,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e40ff61a-5a84-44d4-be7e-3853bfd4dca8}</x14:id>
+          <x14:id>{7c3fd688-a5b1-4984-9ae8-d65cd3b1eb1c}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -422,7 +413,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{358dffa1-56c8-4c78-92b0-c2d4055cbf98}</x14:id>
+          <x14:id>{9ca93616-467e-4e6e-805e-b08fc8d51b65}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -436,7 +427,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e40ff61a-5a84-44d4-be7e-3853bfd4dca8}">
+          <x14:cfRule type="dataBar" id="{7c3fd688-a5b1-4984-9ae8-d65cd3b1eb1c}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -451,7 +442,7 @@
           <xm:sqref>A1:A4</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{358dffa1-56c8-4c78-92b0-c2d4055cbf98}">
+          <x14:cfRule type="dataBar" id="{9ca93616-467e-4e6e-805e-b08fc8d51b65}">
             <x14:dataBar minLength="0" maxLength="100" showValue="0" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>-100</xm:f>

</xml_diff>